<commit_message>
Filigrane des notes chiffrables : mention « NÉANT » seule
Le filigrane calculé des notes chiffrables affichait « NÉANT - NOTE NON
RENSEIGNÉE ». Il n'affiche plus que « NÉANT », en corps 48 (au lieu de 26)
puisque la mention est courte, pour rester lisible comme filigrane.

Le filigrane fixe des notes déclaratives (« NOTE À COMPLÉTER ») est
inchangé.

Les cinq liasses d'exemple et le gabarit vierge sont régénérés. Contrôles
après recalcul : 23/2/20/13/2/20 « doit être 0 » à zéro, trois verdicts
d'équilibre par balance, 0 formule invalide, 0 tiret cadratin. Filigrane
affiché sur 12 notes vides (SN) et 15 (associations), masqué sur les notes
alimentées.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KS6ntrxKkiZTUrYfJS9zZZ
</commit_message>
<xml_diff>
--- a/.claude/skills/sycebnl/liasse/exemples/exemple-etats-projet.xlsx
+++ b/.claude/skills/sycebnl/liasse/exemples/exemple-etats-projet.xlsx
@@ -63,7 +63,7 @@
     <numFmt numFmtId="164" formatCode="_-* #,##0\ _€_-;\-* #,##0\ _€_-;_-* &quot;-&quot;\ _€_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -197,6 +197,12 @@
       <b val="1"/>
       <color rgb="00D9D9D9"/>
       <sz val="26"/>
+    </font>
+    <font>
+      <name val="Arial Black"/>
+      <b val="1"/>
+      <color rgb="00D9D9D9"/>
+      <sz val="48"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -635,7 +641,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="134">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -816,7 +822,7 @@
     <xf numFmtId="164" fontId="6" fillId="6" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -835,7 +841,7 @@
     <xf numFmtId="165" fontId="5" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -848,7 +854,7 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -917,6 +923,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="15"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3594,11 +3603,11 @@
         </is>
       </c>
       <c r="D10" s="5">
-        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"22*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"22*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"292*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"292*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"282*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"282*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2832*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2832*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2931*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2931*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2831*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2831*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2933*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2933*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2932*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2932*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2833*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2833*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2939*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2939*",'BALANCE N'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"22*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"22*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"282*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"282*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"292*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"292*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2933*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2933*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2833*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2833*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2831*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2831*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2931*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2931*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2939*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2939*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2932*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2932*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2832*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2832*",'BALANCE N'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="E10" s="71">
-        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"22*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"22*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"292*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"292*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"282*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"282*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2832*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2832*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2931*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2931*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2831*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2831*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2933*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2933*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2932*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2932*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2833*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2833*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2939*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2939*",'BALANCE N-1'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"22*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"22*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"282*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"282*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"292*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"292*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2933*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2933*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2833*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2833*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2831*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2831*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2931*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2931*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2939*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2939*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2932*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2932*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2832*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2832*",'BALANCE N-1'!$G$2:$G$50)))</f>
         <v/>
       </c>
     </row>
@@ -3619,11 +3628,11 @@
         </is>
       </c>
       <c r="D11" s="5">
-        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"2934*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2934*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2834*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2834*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2838*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2838*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2938*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2938*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2835*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2835*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2935*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2935*",'BALANCE N'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"2834*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2834*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2835*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2835*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2838*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2838*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2938*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2938*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2935*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2935*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2934*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2934*",'BALANCE N'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="E11" s="71">
-        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"2934*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2934*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2834*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2834*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2838*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2838*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2938*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2938*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2835*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2835*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2935*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2935*",'BALANCE N-1'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"2834*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2834*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2835*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2835*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2838*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2838*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2938*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2938*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2935*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2935*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2934*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2934*",'BALANCE N-1'!$G$2:$G$50)))</f>
         <v/>
       </c>
     </row>
@@ -3644,11 +3653,11 @@
         </is>
       </c>
       <c r="D12" s="5">
-        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"24*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"24*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"245*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"245*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2495*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2495*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"294*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"294*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"284*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"284*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2945*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2945*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2845*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2845*",'BALANCE N'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"24*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"24*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"245*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"245*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2495*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2495*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"284*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"284*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"294*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"294*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2845*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2845*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2945*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2945*",'BALANCE N'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="E12" s="71">
-        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"24*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"24*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"245*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"245*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2495*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2495*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"294*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"294*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"284*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"284*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2945*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2945*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2845*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2845*",'BALANCE N-1'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"24*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"24*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"245*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"245*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2495*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2495*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"284*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"284*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"294*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"294*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2845*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2845*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2945*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2945*",'BALANCE N-1'!$G$2:$G$50)))</f>
         <v/>
       </c>
     </row>
@@ -3669,11 +3678,11 @@
         </is>
       </c>
       <c r="D13" s="5">
-        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"245*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"245*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2495*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2495*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"2945*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2945*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2845*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2845*",'BALANCE N'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"245*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"245*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2495*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2495*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"2845*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2845*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2945*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2945*",'BALANCE N'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="E13" s="71">
-        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"245*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"245*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2495*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2495*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"2945*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2945*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2845*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2845*",'BALANCE N-1'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"245*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"245*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2495*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2495*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"2845*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2845*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2945*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2945*",'BALANCE N-1'!$G$2:$G$50)))</f>
         <v/>
       </c>
     </row>
@@ -3744,11 +3753,11 @@
         </is>
       </c>
       <c r="D16" s="5">
-        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"296*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"296*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"297*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"297*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2975*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2975*",'BALANCE N'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"296*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"296*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"297*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"297*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2975*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2975*",'BALANCE N'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="E16" s="71">
-        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"296*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"296*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"297*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"297*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2975*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2975*",'BALANCE N-1'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"296*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"296*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"297*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"297*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2975*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2975*",'BALANCE N-1'!$G$2:$G$50)))</f>
         <v/>
       </c>
     </row>
@@ -3815,11 +3824,11 @@
         </is>
       </c>
       <c r="D19" s="5">
-        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"37*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"37*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"33*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"33*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"38*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"38*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"32*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"32*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"36*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"36*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"34*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"34*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"31*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"31*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"39*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"39*",'BALANCE N'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"34*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"34*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"36*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"36*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"31*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"31*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"32*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"32*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"37*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"37*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"33*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"33*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"38*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"38*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"39*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"39*",'BALANCE N'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="E19" s="71">
-        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"37*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"37*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"33*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"33*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"38*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"38*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"32*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"32*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"36*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"36*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"34*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"34*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"31*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"31*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"39*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"39*",'BALANCE N-1'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"34*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"34*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"36*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"36*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"31*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"31*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"32*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"32*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"37*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"37*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"33*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"33*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"38*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"38*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"39*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"39*",'BALANCE N-1'!$G$2:$G$50)))</f>
         <v/>
       </c>
     </row>
@@ -3890,11 +3899,11 @@
         </is>
       </c>
       <c r="D22" s="5">
-        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"42*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"47*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"43*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"44*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"478*",'BALANCE N'!$G$2:$G$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"44*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"43*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"47*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"42*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"478*",'BALANCE N'!$G$2:$G$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="E22" s="71">
-        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"42*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"47*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"43*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"44*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"478*",'BALANCE N-1'!$G$2:$G$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"44*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"43*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"47*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"42*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"478*",'BALANCE N-1'!$G$2:$G$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$G$2:$G$50)))</f>
         <v/>
       </c>
     </row>
@@ -3961,11 +3970,11 @@
         </is>
       </c>
       <c r="D25" s="5">
-        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"57*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"57*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"52*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"52*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"55*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"55*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"53*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"53*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N'!$A$2:$A$50,"52*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"52*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"57*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"57*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"55*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"55*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"53*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"53*",'BALANCE N'!$H$2:$H$50)))-((SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="E25" s="71">
-        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"57*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"57*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"52*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"52*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"55*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"55*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"53*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"53*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$G$2:$G$50)))</f>
+        <f>((SUMIF('BALANCE N-1'!$A$2:$A$50,"52*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"52*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"57*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"57*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"55*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"55*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"53*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"53*",'BALANCE N-1'!$H$2:$H$50)))-((SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$G$2:$G$50)))</f>
         <v/>
       </c>
     </row>
@@ -4387,11 +4396,11 @@
         </is>
       </c>
       <c r="D18" s="5">
-        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"484*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"484*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"481*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"481*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"481*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"481*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"484*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"484*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$G$2:$G$50))</f>
         <v/>
       </c>
       <c r="E18" s="71">
-        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"484*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"484*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"481*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"481*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"481*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"481*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"484*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"484*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$G$2:$G$50))</f>
         <v/>
       </c>
     </row>
@@ -4462,11 +4471,11 @@
         </is>
       </c>
       <c r="D21" s="5">
-        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"419*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"419*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"479*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"479*",'BALANCE N'!$G$2:$G$50))+(SUMIF('BALANCE N'!$A$2:$A$50,"42*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"47*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"43*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"44*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"479*",'BALANCE N'!$H$2:$H$50))</f>
+        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"419*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"419*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"479*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"479*",'BALANCE N'!$G$2:$G$50))+(SUMIF('BALANCE N'!$A$2:$A$50,"44*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"43*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"47*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"42*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"479*",'BALANCE N'!$H$2:$H$50))</f>
         <v/>
       </c>
       <c r="E21" s="71">
-        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"419*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"419*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"479*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"479*",'BALANCE N-1'!$G$2:$G$50))+(SUMIF('BALANCE N-1'!$A$2:$A$50,"42*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"47*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"43*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"44*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"479*",'BALANCE N-1'!$H$2:$H$50))</f>
+        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"419*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"419*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"479*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"479*",'BALANCE N-1'!$G$2:$G$50))+(SUMIF('BALANCE N-1'!$A$2:$A$50,"44*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"43*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"47*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"42*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"479*",'BALANCE N-1'!$H$2:$H$50))</f>
         <v/>
       </c>
     </row>
@@ -4483,11 +4492,11 @@
       </c>
       <c r="C22" s="104" t="inlineStr"/>
       <c r="D22" s="5">
-        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$G$2:$G$50))</f>
         <v/>
       </c>
       <c r="E22" s="71">
-        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$G$2:$G$50))</f>
         <v/>
       </c>
     </row>
@@ -4825,11 +4834,11 @@
         </is>
       </c>
       <c r="D12" s="5">
-        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"77*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"77*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"72*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"72*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"78*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"78*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"75*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"75*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"73*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"73*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"707*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"707*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"708*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"708*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"706*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"706*",'BALANCE N'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"78*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"78*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"73*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"73*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"77*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"77*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"72*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"72*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"75*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"75*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"706*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"706*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"708*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"708*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"707*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"707*",'BALANCE N'!$G$2:$G$50))</f>
         <v/>
       </c>
       <c r="E12" s="71">
-        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"77*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"77*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"72*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"72*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"78*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"78*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"75*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"75*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"73*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"73*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"707*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"707*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"708*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"708*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"706*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"706*",'BALANCE N-1'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"78*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"78*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"73*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"73*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"77*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"77*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"72*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"72*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"75*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"75*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"706*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"706*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"708*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"708*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"707*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"707*",'BALANCE N-1'!$G$2:$G$50))</f>
         <v/>
       </c>
     </row>
@@ -4896,11 +4905,11 @@
         </is>
       </c>
       <c r="D15" s="5">
-        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"601*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"601*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"602*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"602*",'BALANCE N'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"602*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"602*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"601*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"601*",'BALANCE N'!$G$2:$G$50))</f>
         <v/>
       </c>
       <c r="E15" s="71">
-        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"601*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"601*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"602*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"602*",'BALANCE N-1'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"602*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"602*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"601*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"601*",'BALANCE N-1'!$G$2:$G$50))</f>
         <v/>
       </c>
     </row>
@@ -4921,11 +4930,11 @@
         </is>
       </c>
       <c r="D16" s="5">
-        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"605*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"605*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"604*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"604*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"606*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"606*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"608*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"608*",'BALANCE N'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"608*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"608*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"604*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"604*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"606*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"606*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"605*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"605*",'BALANCE N'!$G$2:$G$50))</f>
         <v/>
       </c>
       <c r="E16" s="71">
-        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"605*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"605*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"604*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"604*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"606*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"606*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"608*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"608*",'BALANCE N-1'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"608*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"608*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"604*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"604*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"606*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"606*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"605*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"605*",'BALANCE N-1'!$G$2:$G$50))</f>
         <v/>
       </c>
     </row>
@@ -5146,11 +5155,11 @@
         </is>
       </c>
       <c r="D25" s="5">
-        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"86*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"86*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"82*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"82*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"84*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"84*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"88*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"88*",'BALANCE N'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"88*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"88*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"82*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"82*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"84*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"84*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"86*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"86*",'BALANCE N'!$G$2:$G$50))</f>
         <v/>
       </c>
       <c r="E25" s="71">
-        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"86*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"86*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"82*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"82*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"84*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"84*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"88*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"88*",'BALANCE N-1'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"88*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"88*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"82*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"82*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"84*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"84*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"86*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"86*",'BALANCE N-1'!$G$2:$G$50))</f>
         <v/>
       </c>
     </row>
@@ -5171,11 +5180,11 @@
         </is>
       </c>
       <c r="D26" s="5">
-        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"85*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"85*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"87*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"87*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"81*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"81*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"83*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"83*",'BALANCE N'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"87*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"87*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"83*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"83*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"81*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"81*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"85*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"85*",'BALANCE N'!$G$2:$G$50))</f>
         <v/>
       </c>
       <c r="E26" s="71">
-        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"85*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"85*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"87*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"87*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"81*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"81*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"83*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"83*",'BALANCE N-1'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N-1'!$A$2:$A$50,"87*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"87*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"83*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"83*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"81*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"81*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"85*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"85*",'BALANCE N-1'!$G$2:$G$50))</f>
         <v/>
       </c>
     </row>
@@ -6433,15 +6442,15 @@
         </is>
       </c>
       <c r="B10" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C10" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"214*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"214*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"212*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"212*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"213*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"213*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"214*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"214*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"213*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"213*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"212*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"212*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="D10" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"214*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"214*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"212*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"212*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"213*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"213*",'BALANCE N'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"214*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"213*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"212*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"214*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"214*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"213*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"213*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"212*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"212*",'BALANCE N'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="E10" s="85">
@@ -6479,15 +6488,15 @@
         </is>
       </c>
       <c r="B12" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C12" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"218*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"218*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"219*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"219*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"219*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"219*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"218*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"218*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="D12" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"218*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"218*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"219*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"219*",'BALANCE N'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"219*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"218*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"219*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"219*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"218*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"218*",'BALANCE N'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="E12" s="85">
@@ -6559,15 +6568,15 @@
         </is>
       </c>
       <c r="B16" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C16" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="D16" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="E16" s="85">
@@ -6582,15 +6591,15 @@
         </is>
       </c>
       <c r="B17" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C17" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="D17" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2315*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2325*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2315*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2325*",'BALANCE N'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="E17" s="85">
@@ -6605,15 +6614,15 @@
         </is>
       </c>
       <c r="B18" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C18" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="D18" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="E18" s="85">
@@ -6731,15 +6740,15 @@
         </is>
       </c>
       <c r="B24" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C24" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="D24" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"275*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"275*",'BALANCE N'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="E24" s="85">
@@ -6794,14 +6803,14 @@
       </c>
     </row>
     <row r="31"/>
-    <row r="32" ht="26" customHeight="1">
-      <c r="A32" s="118">
-        <f>IF(SUM(B9:B25,C9:C25,D9:D25,E9:E25)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="26" customHeight="1"/>
-    <row r="34" ht="26" customHeight="1"/>
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="121">
+        <f>IF(SUM(B9:B25,C9:C25,D9:D25,E9:E25)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="34" customHeight="1"/>
+    <row r="34" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A7:E7"/>
@@ -6901,7 +6910,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="121" t="inlineStr">
+      <c r="A8" s="122" t="inlineStr">
         <is>
           <t>I : crédit-bail immobilier ; M : crédit-bail mobilier ; A : autres contrats</t>
         </is>
@@ -6987,15 +6996,15 @@
         </is>
       </c>
       <c r="B12" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C12" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"2426*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2426*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2416*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2416*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2446*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2446*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"2416*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2416*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2426*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2426*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2446*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2446*",'BALANCE N'!$H$2:$H$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="D12" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"2426*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2426*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2416*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2416*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2446*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2446*",'BALANCE N'!$H$2:$H$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2416*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2426*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2446*",'BALANCE N-1'!$H$2:$H$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"2416*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2416*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2426*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2426*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2446*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2446*",'BALANCE N'!$H$2:$H$50)))</f>
         <v/>
       </c>
       <c r="E12" s="85">
@@ -7073,14 +7082,14 @@
       </c>
     </row>
     <row r="20"/>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="118">
-        <f>IF(SUM(B10:B14,C10:C14,D10:D14,E10:E14)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="26" customHeight="1"/>
-    <row r="23" ht="26" customHeight="1"/>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="121">
+        <f>IF(SUM(B10:B14,C10:C14,D10:D14,E10:E14)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1"/>
+    <row r="23" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A8:E8"/>
@@ -7640,7 +7649,7 @@
       <c r="B9" s="120" t="n"/>
       <c r="C9" s="120" t="n"/>
       <c r="D9" s="120" t="n"/>
-      <c r="E9" s="122" t="n"/>
+      <c r="E9" s="123" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="84" t="inlineStr">
@@ -7660,7 +7669,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -7683,7 +7692,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="124">
+      <c r="E11" s="125">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -7706,7 +7715,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -7725,7 +7734,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="124">
+      <c r="E13" s="125">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -7748,7 +7757,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="124">
+      <c r="E14" s="125">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -7769,7 +7778,7 @@
       <c r="B16" s="120" t="n"/>
       <c r="C16" s="120" t="n"/>
       <c r="D16" s="120" t="n"/>
-      <c r="E16" s="122" t="n"/>
+      <c r="E16" s="123" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="84" t="inlineStr">
@@ -7789,7 +7798,7 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="123">
+      <c r="E17" s="124">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
@@ -7812,7 +7821,7 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="123">
+      <c r="E18" s="124">
         <f>IF(C18=0,"",(B18-C18)/C18)</f>
         <v/>
       </c>
@@ -7835,7 +7844,7 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="124">
+      <c r="E19" s="125">
         <f>IF(C19=0,"",(B19-C19)/C19)</f>
         <v/>
       </c>
@@ -7856,14 +7865,14 @@
       </c>
     </row>
     <row r="23"/>
-    <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="118">
-        <f>IF(SUM(B9:B19,C9:C19,D9:D19)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="26" customHeight="1"/>
-    <row r="26" ht="26" customHeight="1"/>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="121">
+        <f>IF(SUM(B9:B19,C9:C19,D9:D19)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1"/>
+    <row r="26" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A7:E7"/>
@@ -8010,7 +8019,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -8033,7 +8042,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -8056,7 +8065,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -8079,7 +8088,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -8102,7 +8111,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -8125,7 +8134,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -8148,7 +8157,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="123">
+      <c r="E15" s="124">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -8171,7 +8180,7 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="124">
+      <c r="E16" s="125">
         <f>IF(C16=0,"",(B16-C16)/C16)</f>
         <v/>
       </c>
@@ -8194,7 +8203,7 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="123">
+      <c r="E17" s="124">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
@@ -8213,7 +8222,7 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="124">
+      <c r="E18" s="125">
         <f>IF(C18=0,"",(B18-C18)/C18)</f>
         <v/>
       </c>
@@ -8236,20 +8245,20 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="124">
+      <c r="E19" s="125">
         <f>IF(C19=0,"",(B19-C19)/C19)</f>
         <v/>
       </c>
     </row>
     <row r="20"/>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="118">
-        <f>IF(SUM(B9:B19,C9:C19,D9:D19)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="26" customHeight="1"/>
-    <row r="23" ht="26" customHeight="1"/>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="121">
+        <f>IF(SUM(B9:B19,C9:C19,D9:D19)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1"/>
+    <row r="23" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A7:E7"/>
@@ -8414,7 +8423,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -8440,7 +8449,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -8466,7 +8475,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -8492,7 +8501,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -8518,7 +8527,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -8544,7 +8553,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -8570,7 +8579,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="124">
+      <c r="E15" s="125">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -8585,18 +8594,18 @@
         </is>
       </c>
       <c r="B16" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="C16" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="D16" s="85">
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="123">
+      <c r="E16" s="124">
         <f>IF(C16=0,"",(B16-C16)/C16)</f>
         <v/>
       </c>
@@ -8618,7 +8627,7 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="124">
+      <c r="E17" s="125">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
@@ -8644,7 +8653,7 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="124">
+      <c r="E18" s="125">
         <f>IF(C18=0,"",(B18-C18)/C18)</f>
         <v/>
       </c>
@@ -8668,14 +8677,14 @@
       </c>
     </row>
     <row r="22"/>
-    <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="118">
-        <f>IF(SUM(B9:B18,C9:C18,D9:D18,F15:F18,G15:G18,H15:H18)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="26" customHeight="1"/>
-    <row r="25" ht="26" customHeight="1"/>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="121">
+        <f>IF(SUM(B9:B18,C9:C18,D9:D18,F15:F18,G15:G18,H15:H18)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1"/>
+    <row r="25" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A7:H7"/>
@@ -8823,7 +8832,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -8846,7 +8855,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -8869,7 +8878,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -8892,7 +8901,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -8915,7 +8924,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="124">
+      <c r="E13" s="125">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -8938,7 +8947,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -8961,7 +8970,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="123">
+      <c r="E15" s="124">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -8984,7 +8993,7 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="123">
+      <c r="E16" s="124">
         <f>IF(C16=0,"",(B16-C16)/C16)</f>
         <v/>
       </c>
@@ -8996,18 +9005,18 @@
         </is>
       </c>
       <c r="B17" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"523*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"524*",'BALANCE N'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"524*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"523*",'BALANCE N'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="C17" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"523*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"524*",'BALANCE N-1'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"524*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"523*",'BALANCE N-1'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="D17" s="85">
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="123">
+      <c r="E17" s="124">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
@@ -9030,7 +9039,7 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="123">
+      <c r="E18" s="124">
         <f>IF(C18=0,"",(B18-C18)/C18)</f>
         <v/>
       </c>
@@ -9053,7 +9062,7 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="123">
+      <c r="E19" s="124">
         <f>IF(C19=0,"",(B19-C19)/C19)</f>
         <v/>
       </c>
@@ -9065,18 +9074,18 @@
         </is>
       </c>
       <c r="B20" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"532*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"538*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"533*",'BALANCE N'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"533*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"538*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"532*",'BALANCE N'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="C20" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"532*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"538*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"533*",'BALANCE N-1'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"533*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"538*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"532*",'BALANCE N-1'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="D20" s="85">
         <f>B20-C20</f>
         <v/>
       </c>
-      <c r="E20" s="123">
+      <c r="E20" s="124">
         <f>IF(C20=0,"",(B20-C20)/C20)</f>
         <v/>
       </c>
@@ -9099,7 +9108,7 @@
         <f>B21-C21</f>
         <v/>
       </c>
-      <c r="E21" s="123">
+      <c r="E21" s="124">
         <f>IF(C21=0,"",(B21-C21)/C21)</f>
         <v/>
       </c>
@@ -9122,7 +9131,7 @@
         <f>B22-C22</f>
         <v/>
       </c>
-      <c r="E22" s="123">
+      <c r="E22" s="124">
         <f>IF(C22=0,"",(B22-C22)/C22)</f>
         <v/>
       </c>
@@ -9145,7 +9154,7 @@
         <f>B23-C23</f>
         <v/>
       </c>
-      <c r="E23" s="123">
+      <c r="E23" s="124">
         <f>IF(C23=0,"",(B23-C23)/C23)</f>
         <v/>
       </c>
@@ -9168,7 +9177,7 @@
         <f>B24-C24</f>
         <v/>
       </c>
-      <c r="E24" s="124">
+      <c r="E24" s="125">
         <f>IF(C24=0,"",(B24-C24)/C24)</f>
         <v/>
       </c>
@@ -9180,18 +9189,18 @@
         </is>
       </c>
       <c r="B25" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="C25" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="D25" s="85">
         <f>B25-C25</f>
         <v/>
       </c>
-      <c r="E25" s="123">
+      <c r="E25" s="124">
         <f>IF(C25=0,"",(B25-C25)/C25)</f>
         <v/>
       </c>
@@ -9210,7 +9219,7 @@
         <f>B26-C26</f>
         <v/>
       </c>
-      <c r="E26" s="124">
+      <c r="E26" s="125">
         <f>IF(C26=0,"",(B26-C26)/C26)</f>
         <v/>
       </c>
@@ -9233,7 +9242,7 @@
         <f>B27-C27</f>
         <v/>
       </c>
-      <c r="E27" s="124">
+      <c r="E27" s="125">
         <f>IF(C27=0,"",(B27-C27)/C27)</f>
         <v/>
       </c>
@@ -9254,14 +9263,14 @@
       </c>
     </row>
     <row r="31"/>
-    <row r="32" ht="26" customHeight="1">
-      <c r="A32" s="118">
-        <f>IF(SUM(B9:B27,C9:C27,D9:D27)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="26" customHeight="1"/>
-    <row r="34" ht="26" customHeight="1"/>
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="121">
+        <f>IF(SUM(B9:B27,C9:C27,D9:D27)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="34" customHeight="1"/>
+    <row r="34" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A7:E7"/>
@@ -9408,7 +9417,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -9442,7 +9451,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -9459,14 +9468,14 @@
       <c r="E12" s="84" t="n"/>
     </row>
     <row r="13"/>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="118">
-        <f>IF(SUM(B9:B12,C9:C12,D9:D12)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="26" customHeight="1"/>
-    <row r="16" ht="26" customHeight="1"/>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="121">
+        <f>IF(SUM(B9:B12,C9:C12,D9:D12)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1"/>
+    <row r="16" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A7:E7"/>
@@ -9607,17 +9616,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="125" t="inlineStr">
+      <c r="A9" s="126" t="inlineStr">
         <is>
           <t>FONDS D'INVESTISSEMENT</t>
         </is>
       </c>
-      <c r="B9" s="126" t="n"/>
-      <c r="C9" s="126" t="n"/>
-      <c r="D9" s="126" t="n"/>
-      <c r="E9" s="126" t="n"/>
-      <c r="F9" s="126" t="n"/>
-      <c r="G9" s="126" t="n"/>
+      <c r="B9" s="127" t="n"/>
+      <c r="C9" s="127" t="n"/>
+      <c r="D9" s="127" t="n"/>
+      <c r="E9" s="127" t="n"/>
+      <c r="F9" s="127" t="n"/>
+      <c r="G9" s="127" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="84" t="n"/>
@@ -9711,17 +9720,17 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="125" t="inlineStr">
+      <c r="A15" s="126" t="inlineStr">
         <is>
           <t>FONDS D'ADMINISTRATION (2)</t>
         </is>
       </c>
-      <c r="B15" s="126" t="n"/>
-      <c r="C15" s="126" t="n"/>
-      <c r="D15" s="126" t="n"/>
-      <c r="E15" s="126" t="n"/>
-      <c r="F15" s="126" t="n"/>
-      <c r="G15" s="126" t="n"/>
+      <c r="B15" s="127" t="n"/>
+      <c r="C15" s="127" t="n"/>
+      <c r="D15" s="127" t="n"/>
+      <c r="E15" s="127" t="n"/>
+      <c r="F15" s="127" t="n"/>
+      <c r="G15" s="127" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="84" t="n"/>
@@ -9829,7 +9838,7 @@
         </is>
       </c>
       <c r="B23" s="96">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"164*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"164*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"162*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"162*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"163*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"163*",'BALANCE N'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"163*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"163*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"162*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"162*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"164*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"164*",'BALANCE N'!$G$2:$G$50)</f>
         <v/>
       </c>
     </row>
@@ -9840,7 +9849,7 @@
         </is>
       </c>
       <c r="B24" s="96">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"462*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"462*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"464*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"464*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"463*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"463*",'BALANCE N'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"464*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"464*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"463*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"463*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"462*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"462*",'BALANCE N'!$G$2:$G$50)</f>
         <v/>
       </c>
     </row>
@@ -9864,14 +9873,14 @@
       </c>
     </row>
     <row r="28"/>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="118">
-        <f>IF(SUM(B10:B25,C10:C20,D10:D20,E10:E20,F10:F20,G10:G20)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="26" customHeight="1"/>
-    <row r="31" ht="26" customHeight="1"/>
+    <row r="29" ht="34" customHeight="1">
+      <c r="A29" s="121">
+        <f>IF(SUM(B10:B25,C10:C20,D10:D20,E10:E20,F10:F20,G10:G20)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="34" customHeight="1"/>
+    <row r="31" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="F2:G2"/>
@@ -10031,7 +10040,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -10056,7 +10065,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -10081,7 +10090,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -10106,7 +10115,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -10131,7 +10140,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -10156,7 +10165,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -10181,7 +10190,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="123">
+      <c r="E15" s="124">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -10206,7 +10215,7 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="123">
+      <c r="E16" s="124">
         <f>IF(C16=0,"",(B16-C16)/C16)</f>
         <v/>
       </c>
@@ -10231,7 +10240,7 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="124">
+      <c r="E17" s="125">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
@@ -10239,14 +10248,14 @@
       <c r="G17" s="9" t="n"/>
     </row>
     <row r="18"/>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="118">
-        <f>IF(SUM(B9:B17,C9:C17,D9:D17,F17:F17,G17:G17)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="26" customHeight="1"/>
-    <row r="21" ht="26" customHeight="1"/>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="121">
+        <f>IF(SUM(B9:B17,C9:C17,D9:D17,F17:F17,G17:G17)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1"/>
+    <row r="21" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A19:G21"/>
@@ -10412,7 +10421,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -10438,7 +10447,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -10464,7 +10473,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -10490,7 +10499,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -10505,18 +10514,18 @@
         </is>
       </c>
       <c r="B13" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"188*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"188*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"181*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"181*",'BALANCE N'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"181*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"181*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"188*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"188*",'BALANCE N'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="C13" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"188*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"188*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"181*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"181*",'BALANCE N-1'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"181*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"181*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"188*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"188*",'BALANCE N-1'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="D13" s="85">
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -10542,7 +10551,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="124">
+      <c r="E14" s="125">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -10568,7 +10577,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="123">
+      <c r="E15" s="124">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -10594,7 +10603,7 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="123">
+      <c r="E16" s="124">
         <f>IF(C16=0,"",(B16-C16)/C16)</f>
         <v/>
       </c>
@@ -10620,7 +10629,7 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="123">
+      <c r="E17" s="124">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
@@ -10646,7 +10655,7 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="123">
+      <c r="E18" s="124">
         <f>IF(C18=0,"",(B18-C18)/C18)</f>
         <v/>
       </c>
@@ -10661,18 +10670,18 @@
         </is>
       </c>
       <c r="B19" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"187*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"187*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"1876*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"1876*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"1871*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"1871*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"1872*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"1872*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"1873*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"1873*",'BALANCE N'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"187*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"187*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"1871*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"1871*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"1872*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"1872*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"1873*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"1873*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"1876*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"1876*",'BALANCE N'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="C19" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"187*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"187*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"1876*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"1876*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"1871*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"1871*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"1872*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"1872*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"1873*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"1873*",'BALANCE N-1'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"187*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"187*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"1871*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"1871*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"1872*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"1872*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"1873*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"1873*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"1876*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"1876*",'BALANCE N-1'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="D19" s="85">
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="123">
+      <c r="E19" s="124">
         <f>IF(C19=0,"",(B19-C19)/C19)</f>
         <v/>
       </c>
@@ -10698,7 +10707,7 @@
         <f>B20-C20</f>
         <v/>
       </c>
-      <c r="E20" s="124">
+      <c r="E20" s="125">
         <f>IF(C20=0,"",(B20-C20)/C20)</f>
         <v/>
       </c>
@@ -10724,7 +10733,7 @@
         <f>B21-C21</f>
         <v/>
       </c>
-      <c r="E21" s="123">
+      <c r="E21" s="124">
         <f>IF(C21=0,"",(B21-C21)/C21)</f>
         <v/>
       </c>
@@ -10750,7 +10759,7 @@
         <f>B22-C22</f>
         <v/>
       </c>
-      <c r="E22" s="123">
+      <c r="E22" s="124">
         <f>IF(C22=0,"",(B22-C22)/C22)</f>
         <v/>
       </c>
@@ -10776,7 +10785,7 @@
         <f>B23-C23</f>
         <v/>
       </c>
-      <c r="E23" s="123">
+      <c r="E23" s="124">
         <f>IF(C23=0,"",(B23-C23)/C23)</f>
         <v/>
       </c>
@@ -10791,18 +10800,18 @@
         </is>
       </c>
       <c r="B24" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"198*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"198*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"192*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"192*",'BALANCE N'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"192*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"192*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"198*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"198*",'BALANCE N'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="C24" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"198*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"198*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"192*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"192*",'BALANCE N-1'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"192*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"192*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"198*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"198*",'BALANCE N-1'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="D24" s="85">
         <f>B24-C24</f>
         <v/>
       </c>
-      <c r="E24" s="123">
+      <c r="E24" s="124">
         <f>IF(C24=0,"",(B24-C24)/C24)</f>
         <v/>
       </c>
@@ -10828,7 +10837,7 @@
         <f>B25-C25</f>
         <v/>
       </c>
-      <c r="E25" s="124">
+      <c r="E25" s="125">
         <f>IF(C25=0,"",(B25-C25)/C25)</f>
         <v/>
       </c>
@@ -10854,7 +10863,7 @@
         <f>B26-C26</f>
         <v/>
       </c>
-      <c r="E26" s="124">
+      <c r="E26" s="125">
         <f>IF(C26=0,"",(B26-C26)/C26)</f>
         <v/>
       </c>
@@ -10878,14 +10887,14 @@
       </c>
     </row>
     <row r="30"/>
-    <row r="31" ht="26" customHeight="1">
-      <c r="A31" s="118">
-        <f>IF(SUM(B9:B26,C9:C26,D9:D26,F14:F26,G14:G26,H14:H26)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="26" customHeight="1"/>
-    <row r="33" ht="26" customHeight="1"/>
+    <row r="31" ht="34" customHeight="1">
+      <c r="A31" s="121">
+        <f>IF(SUM(B9:B26,C9:C26,D9:D26,F14:F26,G14:G26,H14:H26)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="34" customHeight="1"/>
+    <row r="33" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A7:H7"/>
@@ -11051,7 +11060,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -11077,7 +11086,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -11103,7 +11112,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="124">
+      <c r="E11" s="125">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -11129,7 +11138,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -11155,7 +11164,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -11181,7 +11190,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -11196,18 +11205,18 @@
         </is>
       </c>
       <c r="B15" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"427*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"421*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"428*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"424*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"425*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"423*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"4281*",'BALANCE N'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"425*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"428*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"427*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"424*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"421*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"423*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"4281*",'BALANCE N'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C15" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"427*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"421*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"428*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"424*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"425*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"423*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4281*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"425*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"428*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"427*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"424*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"421*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"423*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4281*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="D15" s="85">
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="123">
+      <c r="E15" s="124">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -11233,7 +11242,7 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="123">
+      <c r="E16" s="124">
         <f>IF(C16=0,"",(B16-C16)/C16)</f>
         <v/>
       </c>
@@ -11259,7 +11268,7 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="123">
+      <c r="E17" s="124">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
@@ -11285,7 +11294,7 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="123">
+      <c r="E18" s="124">
         <f>IF(C18=0,"",(B18-C18)/C18)</f>
         <v/>
       </c>
@@ -11311,7 +11320,7 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="123">
+      <c r="E19" s="124">
         <f>IF(C19=0,"",(B19-C19)/C19)</f>
         <v/>
       </c>
@@ -11337,7 +11346,7 @@
         <f>B20-C20</f>
         <v/>
       </c>
-      <c r="E20" s="123">
+      <c r="E20" s="124">
         <f>IF(C20=0,"",(B20-C20)/C20)</f>
         <v/>
       </c>
@@ -11363,7 +11372,7 @@
         <f>B21-C21</f>
         <v/>
       </c>
-      <c r="E21" s="124">
+      <c r="E21" s="125">
         <f>IF(C21=0,"",(B21-C21)/C21)</f>
         <v/>
       </c>
@@ -11389,7 +11398,7 @@
         <f>B22-C22</f>
         <v/>
       </c>
-      <c r="E22" s="123">
+      <c r="E22" s="124">
         <f>IF(C22=0,"",(B22-C22)/C22)</f>
         <v/>
       </c>
@@ -11404,18 +11413,18 @@
         </is>
       </c>
       <c r="B23" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"445*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"444*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"443*",'BALANCE N'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"444*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"443*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"445*",'BALANCE N'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C23" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"445*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"444*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"443*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"444*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"443*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"445*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="D23" s="85">
         <f>B23-C23</f>
         <v/>
       </c>
-      <c r="E23" s="123">
+      <c r="E23" s="124">
         <f>IF(C23=0,"",(B23-C23)/C23)</f>
         <v/>
       </c>
@@ -11441,7 +11450,7 @@
         <f>B24-C24</f>
         <v/>
       </c>
-      <c r="E24" s="123">
+      <c r="E24" s="124">
         <f>IF(C24=0,"",(B24-C24)/C24)</f>
         <v/>
       </c>
@@ -11456,18 +11465,18 @@
         </is>
       </c>
       <c r="B25" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"448*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"449*",'BALANCE N'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"449*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"448*",'BALANCE N'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C25" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"448*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"449*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"449*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"448*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="D25" s="85">
         <f>B25-C25</f>
         <v/>
       </c>
-      <c r="E25" s="123">
+      <c r="E25" s="124">
         <f>IF(C25=0,"",(B25-C25)/C25)</f>
         <v/>
       </c>
@@ -11493,7 +11502,7 @@
         <f>B26-C26</f>
         <v/>
       </c>
-      <c r="E26" s="124">
+      <c r="E26" s="125">
         <f>IF(C26=0,"",(B26-C26)/C26)</f>
         <v/>
       </c>
@@ -11519,7 +11528,7 @@
         <f>B27-C27</f>
         <v/>
       </c>
-      <c r="E27" s="124">
+      <c r="E27" s="125">
         <f>IF(C27=0,"",(B27-C27)/C27)</f>
         <v/>
       </c>
@@ -11528,14 +11537,14 @@
       <c r="H27" s="9" t="n"/>
     </row>
     <row r="28"/>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="118">
-        <f>IF(SUM(B9:B27,C9:C27,D9:D27,F11:F27,G11:G27,H11:H27)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="26" customHeight="1"/>
-    <row r="31" ht="26" customHeight="1"/>
+    <row r="29" ht="34" customHeight="1">
+      <c r="A29" s="121">
+        <f>IF(SUM(B9:B27,C9:C27,D9:D27,F11:F27,G11:G27,H11:H27)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="34" customHeight="1"/>
+    <row r="31" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A7:H7"/>
@@ -11683,7 +11692,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -11706,7 +11715,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="124">
+      <c r="E10" s="125">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -11729,7 +11738,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -11752,7 +11761,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -11764,18 +11773,18 @@
         </is>
       </c>
       <c r="B13" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"523*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"524*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"525*",'BALANCE N'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"524*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"525*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"523*",'BALANCE N'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C13" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"523*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"524*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"525*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"524*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"525*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"523*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="D13" s="85">
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -11787,18 +11796,18 @@
         </is>
       </c>
       <c r="B14" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"526*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"566*",'BALANCE N'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"566*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"526*",'BALANCE N'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C14" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"526*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"566*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"566*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"526*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="D14" s="85">
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -11821,7 +11830,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="123">
+      <c r="E15" s="124">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -11844,7 +11853,7 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="124">
+      <c r="E16" s="125">
         <f>IF(C16=0,"",(B16-C16)/C16)</f>
         <v/>
       </c>
@@ -11867,20 +11876,20 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="124">
+      <c r="E17" s="125">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
     </row>
     <row r="18"/>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="118">
-        <f>IF(SUM(B9:B17,C9:C17,D9:D17)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="26" customHeight="1"/>
-    <row r="21" ht="26" customHeight="1"/>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="121">
+        <f>IF(SUM(B9:B17,C9:C17,D9:D17)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1"/>
+    <row r="21" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A7:E7"/>
@@ -12238,7 +12247,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -12261,7 +12270,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -12284,7 +12293,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -12307,7 +12316,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -12330,7 +12339,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -12342,18 +12351,18 @@
         </is>
       </c>
       <c r="B14" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"73*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"73*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"78*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"78*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"75*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"75*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"77*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"77*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"708*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"708*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"706*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"706*",'BALANCE N'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"78*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"78*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"73*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"73*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"77*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"77*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"75*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"75*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"706*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"706*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"708*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"708*",'BALANCE N'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="C14" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"73*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"73*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"78*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"78*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"75*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"75*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"77*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"77*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"708*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"708*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"706*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"706*",'BALANCE N-1'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"78*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"78*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"73*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"73*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"77*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"77*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"75*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"75*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"706*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"706*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"708*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"708*",'BALANCE N-1'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="D14" s="85">
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -12376,20 +12385,20 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="124">
+      <c r="E15" s="125">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
     </row>
     <row r="16"/>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="118">
-        <f>IF(SUM(B9:B15,C9:C15,D9:D15)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="26" customHeight="1"/>
-    <row r="19" ht="26" customHeight="1"/>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="121">
+        <f>IF(SUM(B9:B15,C9:C15,D9:D15)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1"/>
+    <row r="19" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A17:E19"/>
@@ -12536,7 +12545,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -12559,7 +12568,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -12582,7 +12591,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -12605,7 +12614,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -12628,7 +12637,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -12651,7 +12660,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -12674,20 +12683,20 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="124">
+      <c r="E15" s="125">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
     </row>
     <row r="16"/>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="118">
-        <f>IF(SUM(B9:B15,C9:C15,D9:D15)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="26" customHeight="1"/>
-    <row r="19" ht="26" customHeight="1"/>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="121">
+        <f>IF(SUM(B9:B15,C9:C15,D9:D15)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1"/>
+    <row r="19" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A17:E19"/>
@@ -12834,7 +12843,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -12857,7 +12866,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -12880,7 +12889,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -12903,7 +12912,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -12926,7 +12935,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -12949,20 +12958,20 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="124">
+      <c r="E14" s="125">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
     </row>
     <row r="15"/>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="118">
-        <f>IF(SUM(B9:B14,C9:C14,D9:D14)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="26" customHeight="1"/>
-    <row r="18" ht="26" customHeight="1"/>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="121">
+        <f>IF(SUM(B9:B14,C9:C14,D9:D14)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1"/>
+    <row r="18" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A7:E7"/>
@@ -13109,7 +13118,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -13132,7 +13141,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -13155,7 +13164,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -13178,7 +13187,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -13201,7 +13210,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -13224,7 +13233,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -13247,7 +13256,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="123">
+      <c r="E15" s="124">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -13270,7 +13279,7 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="123">
+      <c r="E16" s="124">
         <f>IF(C16=0,"",(B16-C16)/C16)</f>
         <v/>
       </c>
@@ -13293,7 +13302,7 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="123">
+      <c r="E17" s="124">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
@@ -13316,7 +13325,7 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="123">
+      <c r="E18" s="124">
         <f>IF(C18=0,"",(B18-C18)/C18)</f>
         <v/>
       </c>
@@ -13339,7 +13348,7 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="123">
+      <c r="E19" s="124">
         <f>IF(C19=0,"",(B19-C19)/C19)</f>
         <v/>
       </c>
@@ -13362,7 +13371,7 @@
         <f>B20-C20</f>
         <v/>
       </c>
-      <c r="E20" s="123">
+      <c r="E20" s="124">
         <f>IF(C20=0,"",(B20-C20)/C20)</f>
         <v/>
       </c>
@@ -13385,7 +13394,7 @@
         <f>B21-C21</f>
         <v/>
       </c>
-      <c r="E21" s="123">
+      <c r="E21" s="124">
         <f>IF(C21=0,"",(B21-C21)/C21)</f>
         <v/>
       </c>
@@ -13408,7 +13417,7 @@
         <f>B22-C22</f>
         <v/>
       </c>
-      <c r="E22" s="123">
+      <c r="E22" s="124">
         <f>IF(C22=0,"",(B22-C22)/C22)</f>
         <v/>
       </c>
@@ -13431,7 +13440,7 @@
         <f>B23-C23</f>
         <v/>
       </c>
-      <c r="E23" s="123">
+      <c r="E23" s="124">
         <f>IF(C23=0,"",(B23-C23)/C23)</f>
         <v/>
       </c>
@@ -13454,7 +13463,7 @@
         <f>B24-C24</f>
         <v/>
       </c>
-      <c r="E24" s="123">
+      <c r="E24" s="124">
         <f>IF(C24=0,"",(B24-C24)/C24)</f>
         <v/>
       </c>
@@ -13477,20 +13486,20 @@
         <f>B25-C25</f>
         <v/>
       </c>
-      <c r="E25" s="124">
+      <c r="E25" s="125">
         <f>IF(C25=0,"",(B25-C25)/C25)</f>
         <v/>
       </c>
     </row>
     <row r="26"/>
-    <row r="27" ht="26" customHeight="1">
-      <c r="A27" s="118">
-        <f>IF(SUM(B9:B25,C9:C25,D9:D25)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="26" customHeight="1"/>
-    <row r="29" ht="26" customHeight="1"/>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="121">
+        <f>IF(SUM(B9:B25,C9:C25,D9:D25)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1"/>
+    <row r="29" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A7:E7"/>
@@ -13637,7 +13646,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -13660,7 +13669,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -13683,7 +13692,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -13706,7 +13715,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -13729,7 +13738,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -13752,7 +13761,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -13775,20 +13784,20 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="124">
+      <c r="E15" s="125">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
     </row>
     <row r="16"/>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="118">
-        <f>IF(SUM(B9:B15,C9:C15,D9:D15)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="26" customHeight="1"/>
-    <row r="19" ht="26" customHeight="1"/>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="121">
+        <f>IF(SUM(B9:B15,C9:C15,D9:D15)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1"/>
+    <row r="19" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A17:E19"/>
@@ -13935,7 +13944,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -13958,7 +13967,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -13981,7 +13990,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -14004,7 +14013,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -14027,7 +14036,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -14050,7 +14059,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -14073,7 +14082,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="124">
+      <c r="E15" s="125">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -14094,14 +14103,14 @@
       </c>
     </row>
     <row r="19"/>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="118">
-        <f>IF(SUM(B9:B15,C9:C15,D9:D15)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="26" customHeight="1"/>
-    <row r="22" ht="26" customHeight="1"/>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="121">
+        <f>IF(SUM(B9:B15,C9:C15,D9:D15)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1"/>
+    <row r="22" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A20:E22"/>
@@ -14248,7 +14257,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -14271,7 +14280,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -14294,7 +14303,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -14317,7 +14326,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -14340,7 +14349,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -14363,7 +14372,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -14386,7 +14395,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="123">
+      <c r="E15" s="124">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -14409,7 +14418,7 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="123">
+      <c r="E16" s="124">
         <f>IF(C16=0,"",(B16-C16)/C16)</f>
         <v/>
       </c>
@@ -14432,20 +14441,20 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="124">
+      <c r="E17" s="125">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
     </row>
     <row r="18"/>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="118">
-        <f>IF(SUM(B9:B17,C9:C17,D9:D17)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="26" customHeight="1"/>
-    <row r="21" ht="26" customHeight="1"/>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="121">
+        <f>IF(SUM(B9:B17,C9:C17,D9:D17)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1"/>
+    <row r="21" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A7:E7"/>
@@ -14775,14 +14784,14 @@
       </c>
     </row>
     <row r="26"/>
-    <row r="27" ht="26" customHeight="1">
-      <c r="A27" s="118">
-        <f>IF(SUM(B24:B24,F10:F14,G10:G14,H10:H14,I10:I14)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="26" customHeight="1"/>
-    <row r="29" ht="26" customHeight="1"/>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="121">
+        <f>IF(SUM(B24:B24,F10:F14,G10:G14,H10:H14,I10:I14)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1"/>
+    <row r="29" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B4:F4"/>
@@ -14930,7 +14939,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -14953,7 +14962,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -14976,7 +14985,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -14999,7 +15008,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -15022,7 +15031,7 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -15045,7 +15054,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -15068,7 +15077,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="123">
+      <c r="E15" s="124">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -15091,7 +15100,7 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="124">
+      <c r="E16" s="125">
         <f>IF(C16=0,"",(B16-C16)/C16)</f>
         <v/>
       </c>
@@ -15114,7 +15123,7 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="123">
+      <c r="E17" s="124">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
@@ -15137,7 +15146,7 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="123">
+      <c r="E18" s="124">
         <f>IF(C18=0,"",(B18-C18)/C18)</f>
         <v/>
       </c>
@@ -15160,7 +15169,7 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="123">
+      <c r="E19" s="124">
         <f>IF(C19=0,"",(B19-C19)/C19)</f>
         <v/>
       </c>
@@ -15183,7 +15192,7 @@
         <f>B20-C20</f>
         <v/>
       </c>
-      <c r="E20" s="123">
+      <c r="E20" s="124">
         <f>IF(C20=0,"",(B20-C20)/C20)</f>
         <v/>
       </c>
@@ -15206,7 +15215,7 @@
         <f>B21-C21</f>
         <v/>
       </c>
-      <c r="E21" s="123">
+      <c r="E21" s="124">
         <f>IF(C21=0,"",(B21-C21)/C21)</f>
         <v/>
       </c>
@@ -15229,7 +15238,7 @@
         <f>B22-C22</f>
         <v/>
       </c>
-      <c r="E22" s="123">
+      <c r="E22" s="124">
         <f>IF(C22=0,"",(B22-C22)/C22)</f>
         <v/>
       </c>
@@ -15252,7 +15261,7 @@
         <f>B23-C23</f>
         <v/>
       </c>
-      <c r="E23" s="123">
+      <c r="E23" s="124">
         <f>IF(C23=0,"",(B23-C23)/C23)</f>
         <v/>
       </c>
@@ -15275,7 +15284,7 @@
         <f>B24-C24</f>
         <v/>
       </c>
-      <c r="E24" s="123">
+      <c r="E24" s="124">
         <f>IF(C24=0,"",(B24-C24)/C24)</f>
         <v/>
       </c>
@@ -15298,7 +15307,7 @@
         <f>B25-C25</f>
         <v/>
       </c>
-      <c r="E25" s="124">
+      <c r="E25" s="125">
         <f>IF(C25=0,"",(B25-C25)/C25)</f>
         <v/>
       </c>
@@ -15321,20 +15330,20 @@
         <f>B26-C26</f>
         <v/>
       </c>
-      <c r="E26" s="124">
+      <c r="E26" s="125">
         <f>IF(C26=0,"",(B26-C26)/C26)</f>
         <v/>
       </c>
     </row>
     <row r="27"/>
-    <row r="28" ht="26" customHeight="1">
-      <c r="A28" s="118">
-        <f>IF(SUM(B9:B26,C9:C26,D9:D26)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="26" customHeight="1"/>
-    <row r="30" ht="26" customHeight="1"/>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="121">
+        <f>IF(SUM(B9:B26,C9:C26,D9:D26)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1"/>
+    <row r="30" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A28:E30"/>
@@ -15615,17 +15624,17 @@
         </is>
       </c>
       <c r="B13" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="C13" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$G$2:$G$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$G$2:$G$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$G$2:$G$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="D13" s="85" t="n"/>
       <c r="E13" s="85" t="n"/>
       <c r="F13" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$G$2:$G$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$G$2:$G$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"493*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"497*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"490*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"492*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"494*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"491*",'BALANCE N-1'!$G$2:$G$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"493*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"497*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"490*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"492*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"494*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"491*",'BALANCE N'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="G13" s="85" t="n"/>
@@ -15669,18 +15678,18 @@
         </is>
       </c>
       <c r="B15" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="C15" s="85" t="n"/>
       <c r="D15" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$G$2:$G$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$G$2:$G$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$G$2:$G$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="E15" s="85" t="n"/>
       <c r="F15" s="85" t="n"/>
       <c r="G15" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$G$2:$G$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$G$2:$G$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"592*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"591*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"595*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"593*",'BALANCE N-1'!$G$2:$G$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"592*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"591*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"595*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"593*",'BALANCE N'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="H15" s="85" t="n"/>
@@ -15696,17 +15705,17 @@
         </is>
       </c>
       <c r="B16" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$G$2:$G$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$G$2:$G$50)</f>
         <v/>
       </c>
       <c r="C16" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$G$2:$G$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$G$2:$G$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$G$2:$G$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="D16" s="85" t="n"/>
       <c r="E16" s="85" t="n"/>
       <c r="F16" s="85">
-        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$G$2:$G$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$G$2:$G$50)))</f>
+        <f>MAX(0,(SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"499*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"599*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"4998*",'BALANCE N-1'!$G$2:$G$50))-(SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"499*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"599*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"4998*",'BALANCE N'!$G$2:$G$50)))</f>
         <v/>
       </c>
       <c r="G16" s="85" t="n"/>
@@ -15803,14 +15812,14 @@
       </c>
     </row>
     <row r="21"/>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="118">
-        <f>IF(SUM(B9:B18,C9:C18,D9:D18,E9:E18,F9:F18,G9:G18,H9:H18,I9:I18)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="26" customHeight="1"/>
-    <row r="24" ht="26" customHeight="1"/>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="121">
+        <f>IF(SUM(B9:B18,C9:C18,D9:D18,E9:E18,F9:F18,G9:G18,H9:H18,I9:I18)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1"/>
+    <row r="24" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B4:F4"/>
@@ -16271,7 +16280,7 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="123">
+      <c r="E9" s="124">
         <f>IF(C9=0,"",(B9-C9)/C9)</f>
         <v/>
       </c>
@@ -16294,7 +16303,7 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="123">
+      <c r="E10" s="124">
         <f>IF(C10=0,"",(B10-C10)/C10)</f>
         <v/>
       </c>
@@ -16317,7 +16326,7 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="123">
+      <c r="E11" s="124">
         <f>IF(C11=0,"",(B11-C11)/C11)</f>
         <v/>
       </c>
@@ -16340,7 +16349,7 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="124">
         <f>IF(C12=0,"",(B12-C12)/C12)</f>
         <v/>
       </c>
@@ -16352,18 +16361,18 @@
         </is>
       </c>
       <c r="B13" s="85">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"839*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"839*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"838*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"838*",'BALANCE N'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"838*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"838*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"839*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"839*",'BALANCE N'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="C13" s="85">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"839*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"839*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"838*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"838*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"838*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"838*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"839*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"839*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="D13" s="85">
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="123">
+      <c r="E13" s="124">
         <f>IF(C13=0,"",(B13-C13)/C13)</f>
         <v/>
       </c>
@@ -16386,7 +16395,7 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="123">
+      <c r="E14" s="124">
         <f>IF(C14=0,"",(B14-C14)/C14)</f>
         <v/>
       </c>
@@ -16409,7 +16418,7 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="123">
+      <c r="E15" s="124">
         <f>IF(C15=0,"",(B15-C15)/C15)</f>
         <v/>
       </c>
@@ -16432,7 +16441,7 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="123">
+      <c r="E16" s="124">
         <f>IF(C16=0,"",(B16-C16)/C16)</f>
         <v/>
       </c>
@@ -16455,7 +16464,7 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="124">
+      <c r="E17" s="125">
         <f>IF(C17=0,"",(B17-C17)/C17)</f>
         <v/>
       </c>
@@ -16478,7 +16487,7 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="123">
+      <c r="E18" s="124">
         <f>IF(C18=0,"",(B18-C18)/C18)</f>
         <v/>
       </c>
@@ -16501,7 +16510,7 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="123">
+      <c r="E19" s="124">
         <f>IF(C19=0,"",(B19-C19)/C19)</f>
         <v/>
       </c>
@@ -16524,7 +16533,7 @@
         <f>B20-C20</f>
         <v/>
       </c>
-      <c r="E20" s="123">
+      <c r="E20" s="124">
         <f>IF(C20=0,"",(B20-C20)/C20)</f>
         <v/>
       </c>
@@ -16547,7 +16556,7 @@
         <f>B21-C21</f>
         <v/>
       </c>
-      <c r="E21" s="123">
+      <c r="E21" s="124">
         <f>IF(C21=0,"",(B21-C21)/C21)</f>
         <v/>
       </c>
@@ -16570,7 +16579,7 @@
         <f>B22-C22</f>
         <v/>
       </c>
-      <c r="E22" s="123">
+      <c r="E22" s="124">
         <f>IF(C22=0,"",(B22-C22)/C22)</f>
         <v/>
       </c>
@@ -16593,7 +16602,7 @@
         <f>B23-C23</f>
         <v/>
       </c>
-      <c r="E23" s="123">
+      <c r="E23" s="124">
         <f>IF(C23=0,"",(B23-C23)/C23)</f>
         <v/>
       </c>
@@ -16616,7 +16625,7 @@
         <f>B24-C24</f>
         <v/>
       </c>
-      <c r="E24" s="123">
+      <c r="E24" s="124">
         <f>IF(C24=0,"",(B24-C24)/C24)</f>
         <v/>
       </c>
@@ -16639,7 +16648,7 @@
         <f>B25-C25</f>
         <v/>
       </c>
-      <c r="E25" s="123">
+      <c r="E25" s="124">
         <f>IF(C25=0,"",(B25-C25)/C25)</f>
         <v/>
       </c>
@@ -16662,7 +16671,7 @@
         <f>B26-C26</f>
         <v/>
       </c>
-      <c r="E26" s="123">
+      <c r="E26" s="124">
         <f>IF(C26=0,"",(B26-C26)/C26)</f>
         <v/>
       </c>
@@ -16685,7 +16694,7 @@
         <f>B27-C27</f>
         <v/>
       </c>
-      <c r="E27" s="124">
+      <c r="E27" s="125">
         <f>IF(C27=0,"",(B27-C27)/C27)</f>
         <v/>
       </c>
@@ -16708,20 +16717,20 @@
         <f>B28-C28</f>
         <v/>
       </c>
-      <c r="E28" s="124">
+      <c r="E28" s="125">
         <f>IF(C28=0,"",(B28-C28)/C28)</f>
         <v/>
       </c>
     </row>
     <row r="29"/>
-    <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="118">
-        <f>IF(SUM(B9:B28,C9:C28,D9:D28)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="26" customHeight="1"/>
-    <row r="32" ht="26" customHeight="1"/>
+    <row r="30" ht="34" customHeight="1">
+      <c r="A30" s="121">
+        <f>IF(SUM(B9:B28,C9:C28,D9:D28)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="34" customHeight="1"/>
+    <row r="32" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A7:E7"/>
@@ -16882,7 +16891,7 @@
         <f>C9-F9</f>
         <v/>
       </c>
-      <c r="H9" s="123">
+      <c r="H9" s="124">
         <f>IF(C9=0,"",F9/C9)</f>
         <v/>
       </c>
@@ -16901,7 +16910,7 @@
         <f>C10-F10</f>
         <v/>
       </c>
-      <c r="H10" s="123">
+      <c r="H10" s="124">
         <f>IF(C10=0,"",F10/C10)</f>
         <v/>
       </c>
@@ -16920,7 +16929,7 @@
         <f>C11-F11</f>
         <v/>
       </c>
-      <c r="H11" s="123">
+      <c r="H11" s="124">
         <f>IF(C11=0,"",F11/C11)</f>
         <v/>
       </c>
@@ -16939,7 +16948,7 @@
         <f>C12-F12</f>
         <v/>
       </c>
-      <c r="H12" s="123">
+      <c r="H12" s="124">
         <f>IF(C12=0,"",F12/C12)</f>
         <v/>
       </c>
@@ -16958,7 +16967,7 @@
         <f>C13-F13</f>
         <v/>
       </c>
-      <c r="H13" s="123">
+      <c r="H13" s="124">
         <f>IF(C13=0,"",F13/C13)</f>
         <v/>
       </c>
@@ -16977,7 +16986,7 @@
         <f>C14-F14</f>
         <v/>
       </c>
-      <c r="H14" s="123">
+      <c r="H14" s="124">
         <f>IF(C14=0,"",F14/C14)</f>
         <v/>
       </c>
@@ -16996,7 +17005,7 @@
         <f>C15-F15</f>
         <v/>
       </c>
-      <c r="H15" s="123">
+      <c r="H15" s="124">
         <f>IF(C15=0,"",F15/C15)</f>
         <v/>
       </c>
@@ -17015,7 +17024,7 @@
         <f>C16-F16</f>
         <v/>
       </c>
-      <c r="H16" s="123">
+      <c r="H16" s="124">
         <f>IF(C16=0,"",F16/C16)</f>
         <v/>
       </c>
@@ -17034,7 +17043,7 @@
         <f>C17-F17</f>
         <v/>
       </c>
-      <c r="H17" s="123">
+      <c r="H17" s="124">
         <f>IF(C17=0,"",F17/C17)</f>
         <v/>
       </c>
@@ -17053,7 +17062,7 @@
         <f>C18-F18</f>
         <v/>
       </c>
-      <c r="H18" s="123">
+      <c r="H18" s="124">
         <f>IF(C18=0,"",F18/C18)</f>
         <v/>
       </c>
@@ -17072,7 +17081,7 @@
         <f>C19-F19</f>
         <v/>
       </c>
-      <c r="H19" s="123">
+      <c r="H19" s="124">
         <f>IF(C19=0,"",F19/C19)</f>
         <v/>
       </c>
@@ -17091,7 +17100,7 @@
         <f>C20-F20</f>
         <v/>
       </c>
-      <c r="H20" s="123">
+      <c r="H20" s="124">
         <f>IF(C20=0,"",F20/C20)</f>
         <v/>
       </c>
@@ -17123,7 +17132,7 @@
         <f>SUM(G9:G20)</f>
         <v/>
       </c>
-      <c r="H21" s="127">
+      <c r="H21" s="128">
         <f>IF(C21=0,"",F21/C21)</f>
         <v/>
       </c>
@@ -17137,14 +17146,14 @@
       </c>
     </row>
     <row r="24"/>
-    <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="118">
-        <f>IF(SUM(C9:C21,D9:D21,E9:E21,F9:F21,G9:G21)=0,"NÉANT - NOTE NON RENSEIGNÉE","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="26" customHeight="1"/>
-    <row r="27" ht="26" customHeight="1"/>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="121">
+        <f>IF(SUM(C9:C21,D9:D21,E9:E21,F9:F21,G9:G21)=0,"NÉANT","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1"/>
+    <row r="27" ht="34" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A7:H7"/>
@@ -17181,7 +17190,7 @@
           <t>TABLE DES COMMENTAIRES</t>
         </is>
       </c>
-      <c r="G1" s="128" t="inlineStr">
+      <c r="G1" s="129" t="inlineStr">
         <is>
           <t>COMMENTAIRES
 PAGE 1/7</t>
@@ -17233,26 +17242,26 @@
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="129" t="inlineStr">
+      <c r="A6" s="130" t="inlineStr">
         <is>
           <t>Partie 1 : Informations générales</t>
         </is>
       </c>
-      <c r="B6" s="130" t="n"/>
-      <c r="C6" s="130" t="n"/>
-      <c r="D6" s="130" t="n"/>
-      <c r="E6" s="130" t="n"/>
-      <c r="F6" s="130" t="n"/>
-      <c r="G6" s="130" t="n"/>
-      <c r="H6" s="130" t="n"/>
+      <c r="B6" s="131" t="n"/>
+      <c r="C6" s="131" t="n"/>
+      <c r="D6" s="131" t="n"/>
+      <c r="E6" s="131" t="n"/>
+      <c r="F6" s="131" t="n"/>
+      <c r="G6" s="131" t="n"/>
+      <c r="H6" s="131" t="n"/>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="131" t="inlineStr">
+      <c r="A7" s="132" t="inlineStr">
         <is>
           <t>Note 1</t>
         </is>
       </c>
-      <c r="B7" s="132" t="inlineStr">
+      <c r="B7" s="133" t="inlineStr">
         <is>
           <t>INFORMATIONS OBLIGATOIRES</t>
         </is>
@@ -17265,7 +17274,7 @@
       <c r="H7" s="49" t="n"/>
     </row>
     <row r="8" ht="110" customHeight="1">
-      <c r="A8" s="133" t="n"/>
+      <c r="A8" s="134" t="n"/>
       <c r="B8" s="49" t="n"/>
       <c r="C8" s="49" t="n"/>
       <c r="D8" s="49" t="n"/>
@@ -17275,26 +17284,26 @@
       <c r="H8" s="49" t="n"/>
     </row>
     <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="129" t="inlineStr">
+      <c r="A9" s="130" t="inlineStr">
         <is>
           <t>Partie 2 : Notes sur le tableau emplois-ressources, le tableau d'exécution budgétaire et la réconciliation de trésorerie</t>
         </is>
       </c>
-      <c r="B9" s="130" t="n"/>
-      <c r="C9" s="130" t="n"/>
-      <c r="D9" s="130" t="n"/>
-      <c r="E9" s="130" t="n"/>
-      <c r="F9" s="130" t="n"/>
-      <c r="G9" s="130" t="n"/>
-      <c r="H9" s="130" t="n"/>
+      <c r="B9" s="131" t="n"/>
+      <c r="C9" s="131" t="n"/>
+      <c r="D9" s="131" t="n"/>
+      <c r="E9" s="131" t="n"/>
+      <c r="F9" s="131" t="n"/>
+      <c r="G9" s="131" t="n"/>
+      <c r="H9" s="131" t="n"/>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="131" t="inlineStr">
+      <c r="A10" s="132" t="inlineStr">
         <is>
           <t>Note 2</t>
         </is>
       </c>
-      <c r="B10" s="132" t="inlineStr">
+      <c r="B10" s="133" t="inlineStr">
         <is>
           <t>INFORMATIONS SPÉCIFIQUES</t>
         </is>
@@ -17307,7 +17316,7 @@
       <c r="H10" s="49" t="n"/>
     </row>
     <row r="11" ht="110" customHeight="1">
-      <c r="A11" s="133" t="n"/>
+      <c r="A11" s="134" t="n"/>
       <c r="B11" s="49" t="n"/>
       <c r="C11" s="49" t="n"/>
       <c r="D11" s="49" t="n"/>
@@ -17317,26 +17326,26 @@
       <c r="H11" s="49" t="n"/>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="129" t="inlineStr">
+      <c r="A12" s="130" t="inlineStr">
         <is>
           <t>Partie 3 : Notes sur le bilan</t>
         </is>
       </c>
-      <c r="B12" s="130" t="n"/>
-      <c r="C12" s="130" t="n"/>
-      <c r="D12" s="130" t="n"/>
-      <c r="E12" s="130" t="n"/>
-      <c r="F12" s="130" t="n"/>
-      <c r="G12" s="130" t="n"/>
-      <c r="H12" s="130" t="n"/>
+      <c r="B12" s="131" t="n"/>
+      <c r="C12" s="131" t="n"/>
+      <c r="D12" s="131" t="n"/>
+      <c r="E12" s="131" t="n"/>
+      <c r="F12" s="131" t="n"/>
+      <c r="G12" s="131" t="n"/>
+      <c r="H12" s="131" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="131" t="inlineStr">
+      <c r="A13" s="132" t="inlineStr">
         <is>
           <t>Note 3A</t>
         </is>
       </c>
-      <c r="B13" s="132" t="inlineStr">
+      <c r="B13" s="133" t="inlineStr">
         <is>
           <t>IMMOBILISATIONS BRUTES</t>
         </is>
@@ -17349,7 +17358,7 @@
       <c r="H13" s="49" t="n"/>
     </row>
     <row r="14" ht="110" customHeight="1">
-      <c r="A14" s="133" t="n"/>
+      <c r="A14" s="134" t="n"/>
       <c r="B14" s="49" t="n"/>
       <c r="C14" s="49" t="n"/>
       <c r="D14" s="49" t="n"/>
@@ -17359,12 +17368,12 @@
       <c r="H14" s="49" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="131" t="inlineStr">
+      <c r="A15" s="132" t="inlineStr">
         <is>
           <t>Note 3B</t>
         </is>
       </c>
-      <c r="B15" s="132" t="inlineStr">
+      <c r="B15" s="133" t="inlineStr">
         <is>
           <t>BIENS PRIS EN LOCATION-ACQUISITION</t>
         </is>
@@ -17377,7 +17386,7 @@
       <c r="H15" s="49" t="n"/>
     </row>
     <row r="16" ht="110" customHeight="1">
-      <c r="A16" s="133" t="n"/>
+      <c r="A16" s="134" t="n"/>
       <c r="B16" s="49" t="n"/>
       <c r="C16" s="49" t="n"/>
       <c r="D16" s="49" t="n"/>
@@ -17392,7 +17401,7 @@
           <t>TABLE DES COMMENTAIRES</t>
         </is>
       </c>
-      <c r="G17" s="128" t="inlineStr">
+      <c r="G17" s="129" t="inlineStr">
         <is>
           <t>COMMENTAIRES
 PAGE 2/7</t>
@@ -17444,12 +17453,12 @@
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="131" t="inlineStr">
+      <c r="A22" s="132" t="inlineStr">
         <is>
           <t>Note 4</t>
         </is>
       </c>
-      <c r="B22" s="132" t="inlineStr">
+      <c r="B22" s="133" t="inlineStr">
         <is>
           <t>ACTIF CIRCULANT ET DETTES CIRCULANTES HAO</t>
         </is>
@@ -17462,7 +17471,7 @@
       <c r="H22" s="49" t="n"/>
     </row>
     <row r="23" ht="110" customHeight="1">
-      <c r="A23" s="133" t="n"/>
+      <c r="A23" s="134" t="n"/>
       <c r="B23" s="49" t="n"/>
       <c r="C23" s="49" t="n"/>
       <c r="D23" s="49" t="n"/>
@@ -17472,12 +17481,12 @@
       <c r="H23" s="49" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="131" t="inlineStr">
+      <c r="A24" s="132" t="inlineStr">
         <is>
           <t>Note 5</t>
         </is>
       </c>
-      <c r="B24" s="132" t="inlineStr">
+      <c r="B24" s="133" t="inlineStr">
         <is>
           <t>STOCKS ET ENCOURS</t>
         </is>
@@ -17490,7 +17499,7 @@
       <c r="H24" s="49" t="n"/>
     </row>
     <row r="25" ht="110" customHeight="1">
-      <c r="A25" s="133" t="n"/>
+      <c r="A25" s="134" t="n"/>
       <c r="B25" s="49" t="n"/>
       <c r="C25" s="49" t="n"/>
       <c r="D25" s="49" t="n"/>
@@ -17500,12 +17509,12 @@
       <c r="H25" s="49" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="131" t="inlineStr">
+      <c r="A26" s="132" t="inlineStr">
         <is>
           <t>Note 6</t>
         </is>
       </c>
-      <c r="B26" s="132" t="inlineStr">
+      <c r="B26" s="133" t="inlineStr">
         <is>
           <t>CLIENTS-USAGERS ET AUTRES CRÉANCES</t>
         </is>
@@ -17518,7 +17527,7 @@
       <c r="H26" s="49" t="n"/>
     </row>
     <row r="27" ht="110" customHeight="1">
-      <c r="A27" s="133" t="n"/>
+      <c r="A27" s="134" t="n"/>
       <c r="B27" s="49" t="n"/>
       <c r="C27" s="49" t="n"/>
       <c r="D27" s="49" t="n"/>
@@ -17528,12 +17537,12 @@
       <c r="H27" s="49" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="131" t="inlineStr">
+      <c r="A28" s="132" t="inlineStr">
         <is>
           <t>Note 7</t>
         </is>
       </c>
-      <c r="B28" s="132" t="inlineStr">
+      <c r="B28" s="133" t="inlineStr">
         <is>
           <t>DISPONIBILITÉS</t>
         </is>
@@ -17546,7 +17555,7 @@
       <c r="H28" s="49" t="n"/>
     </row>
     <row r="29" ht="110" customHeight="1">
-      <c r="A29" s="133" t="n"/>
+      <c r="A29" s="134" t="n"/>
       <c r="B29" s="49" t="n"/>
       <c r="C29" s="49" t="n"/>
       <c r="D29" s="49" t="n"/>
@@ -17561,7 +17570,7 @@
           <t>TABLE DES COMMENTAIRES</t>
         </is>
       </c>
-      <c r="G30" s="128" t="inlineStr">
+      <c r="G30" s="129" t="inlineStr">
         <is>
           <t>COMMENTAIRES
 PAGE 3/7</t>
@@ -17613,12 +17622,12 @@
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="131" t="inlineStr">
+      <c r="A35" s="132" t="inlineStr">
         <is>
           <t>Note 8</t>
         </is>
       </c>
-      <c r="B35" s="132" t="inlineStr">
+      <c r="B35" s="133" t="inlineStr">
         <is>
           <t>ÉCARTS DE CONVERSION</t>
         </is>
@@ -17631,7 +17640,7 @@
       <c r="H35" s="49" t="n"/>
     </row>
     <row r="36" ht="110" customHeight="1">
-      <c r="A36" s="133" t="n"/>
+      <c r="A36" s="134" t="n"/>
       <c r="B36" s="49" t="n"/>
       <c r="C36" s="49" t="n"/>
       <c r="D36" s="49" t="n"/>
@@ -17641,12 +17650,12 @@
       <c r="H36" s="49" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="131" t="inlineStr">
+      <c r="A37" s="132" t="inlineStr">
         <is>
           <t>Note 9</t>
         </is>
       </c>
-      <c r="B37" s="132" t="inlineStr">
+      <c r="B37" s="133" t="inlineStr">
         <is>
           <t>FONDS DU BAILLEUR</t>
         </is>
@@ -17659,7 +17668,7 @@
       <c r="H37" s="49" t="n"/>
     </row>
     <row r="38" ht="110" customHeight="1">
-      <c r="A38" s="133" t="n"/>
+      <c r="A38" s="134" t="n"/>
       <c r="B38" s="49" t="n"/>
       <c r="C38" s="49" t="n"/>
       <c r="D38" s="49" t="n"/>
@@ -17669,12 +17678,12 @@
       <c r="H38" s="49" t="n"/>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="131" t="inlineStr">
+      <c r="A39" s="132" t="inlineStr">
         <is>
           <t>Note 10</t>
         </is>
       </c>
-      <c r="B39" s="132" t="inlineStr">
+      <c r="B39" s="133" t="inlineStr">
         <is>
           <t>SUBVENTIONS</t>
         </is>
@@ -17687,7 +17696,7 @@
       <c r="H39" s="49" t="n"/>
     </row>
     <row r="40" ht="110" customHeight="1">
-      <c r="A40" s="133" t="n"/>
+      <c r="A40" s="134" t="n"/>
       <c r="B40" s="49" t="n"/>
       <c r="C40" s="49" t="n"/>
       <c r="D40" s="49" t="n"/>
@@ -17697,12 +17706,12 @@
       <c r="H40" s="49" t="n"/>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="131" t="inlineStr">
+      <c r="A41" s="132" t="inlineStr">
         <is>
           <t>Note 11</t>
         </is>
       </c>
-      <c r="B41" s="132" t="inlineStr">
+      <c r="B41" s="133" t="inlineStr">
         <is>
           <t>DETTES FINANCIÈRES ET RESSOURCES ASSIMILÉES</t>
         </is>
@@ -17715,7 +17724,7 @@
       <c r="H41" s="49" t="n"/>
     </row>
     <row r="42" ht="110" customHeight="1">
-      <c r="A42" s="133" t="n"/>
+      <c r="A42" s="134" t="n"/>
       <c r="B42" s="49" t="n"/>
       <c r="C42" s="49" t="n"/>
       <c r="D42" s="49" t="n"/>
@@ -17730,7 +17739,7 @@
           <t>TABLE DES COMMENTAIRES</t>
         </is>
       </c>
-      <c r="G43" s="128" t="inlineStr">
+      <c r="G43" s="129" t="inlineStr">
         <is>
           <t>COMMENTAIRES
 PAGE 4/7</t>
@@ -17782,12 +17791,12 @@
       </c>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="131" t="inlineStr">
+      <c r="A48" s="132" t="inlineStr">
         <is>
           <t>Note 12</t>
         </is>
       </c>
-      <c r="B48" s="132" t="inlineStr">
+      <c r="B48" s="133" t="inlineStr">
         <is>
           <t>DETTES FOURNISSEURS ET ASSIMILÉES, FISCALES ET SOCIALES</t>
         </is>
@@ -17800,7 +17809,7 @@
       <c r="H48" s="49" t="n"/>
     </row>
     <row r="49" ht="110" customHeight="1">
-      <c r="A49" s="133" t="n"/>
+      <c r="A49" s="134" t="n"/>
       <c r="B49" s="49" t="n"/>
       <c r="C49" s="49" t="n"/>
       <c r="D49" s="49" t="n"/>
@@ -17810,12 +17819,12 @@
       <c r="H49" s="49" t="n"/>
     </row>
     <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="131" t="inlineStr">
+      <c r="A50" s="132" t="inlineStr">
         <is>
           <t>Note 13</t>
         </is>
       </c>
-      <c r="B50" s="132" t="inlineStr">
+      <c r="B50" s="133" t="inlineStr">
         <is>
           <t>BANQUES, CRÉDIT D'ESCOMPTE ET DE TRÉSORERIE</t>
         </is>
@@ -17828,7 +17837,7 @@
       <c r="H50" s="49" t="n"/>
     </row>
     <row r="51" ht="110" customHeight="1">
-      <c r="A51" s="133" t="n"/>
+      <c r="A51" s="134" t="n"/>
       <c r="B51" s="49" t="n"/>
       <c r="C51" s="49" t="n"/>
       <c r="D51" s="49" t="n"/>
@@ -17838,26 +17847,26 @@
       <c r="H51" s="49" t="n"/>
     </row>
     <row r="52" ht="17" customHeight="1">
-      <c r="A52" s="129" t="inlineStr">
+      <c r="A52" s="130" t="inlineStr">
         <is>
           <t>Partie 4 : Notes sur le compte d'exploitation</t>
         </is>
       </c>
-      <c r="B52" s="130" t="n"/>
-      <c r="C52" s="130" t="n"/>
-      <c r="D52" s="130" t="n"/>
-      <c r="E52" s="130" t="n"/>
-      <c r="F52" s="130" t="n"/>
-      <c r="G52" s="130" t="n"/>
-      <c r="H52" s="130" t="n"/>
+      <c r="B52" s="131" t="n"/>
+      <c r="C52" s="131" t="n"/>
+      <c r="D52" s="131" t="n"/>
+      <c r="E52" s="131" t="n"/>
+      <c r="F52" s="131" t="n"/>
+      <c r="G52" s="131" t="n"/>
+      <c r="H52" s="131" t="n"/>
     </row>
     <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="131" t="inlineStr">
+      <c r="A53" s="132" t="inlineStr">
         <is>
           <t>Note 14</t>
         </is>
       </c>
-      <c r="B53" s="132" t="inlineStr">
+      <c r="B53" s="133" t="inlineStr">
         <is>
           <t>REVENUS ET AUTRES PRODUITS</t>
         </is>
@@ -17870,7 +17879,7 @@
       <c r="H53" s="49" t="n"/>
     </row>
     <row r="54" ht="110" customHeight="1">
-      <c r="A54" s="133" t="n"/>
+      <c r="A54" s="134" t="n"/>
       <c r="B54" s="49" t="n"/>
       <c r="C54" s="49" t="n"/>
       <c r="D54" s="49" t="n"/>
@@ -17880,12 +17889,12 @@
       <c r="H54" s="49" t="n"/>
     </row>
     <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="131" t="inlineStr">
+      <c r="A55" s="132" t="inlineStr">
         <is>
           <t>Note 15</t>
         </is>
       </c>
-      <c r="B55" s="132" t="inlineStr">
+      <c r="B55" s="133" t="inlineStr">
         <is>
           <t>ACHATS</t>
         </is>
@@ -17898,7 +17907,7 @@
       <c r="H55" s="49" t="n"/>
     </row>
     <row r="56" ht="110" customHeight="1">
-      <c r="A56" s="133" t="n"/>
+      <c r="A56" s="134" t="n"/>
       <c r="B56" s="49" t="n"/>
       <c r="C56" s="49" t="n"/>
       <c r="D56" s="49" t="n"/>
@@ -17913,7 +17922,7 @@
           <t>TABLE DES COMMENTAIRES</t>
         </is>
       </c>
-      <c r="G57" s="128" t="inlineStr">
+      <c r="G57" s="129" t="inlineStr">
         <is>
           <t>COMMENTAIRES
 PAGE 5/7</t>
@@ -17965,12 +17974,12 @@
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
-      <c r="A62" s="131" t="inlineStr">
+      <c r="A62" s="132" t="inlineStr">
         <is>
           <t>Note 16</t>
         </is>
       </c>
-      <c r="B62" s="132" t="inlineStr">
+      <c r="B62" s="133" t="inlineStr">
         <is>
           <t>TRANSPORTS</t>
         </is>
@@ -17983,7 +17992,7 @@
       <c r="H62" s="49" t="n"/>
     </row>
     <row r="63" ht="110" customHeight="1">
-      <c r="A63" s="133" t="n"/>
+      <c r="A63" s="134" t="n"/>
       <c r="B63" s="49" t="n"/>
       <c r="C63" s="49" t="n"/>
       <c r="D63" s="49" t="n"/>
@@ -17993,12 +18002,12 @@
       <c r="H63" s="49" t="n"/>
     </row>
     <row r="64" ht="16" customHeight="1">
-      <c r="A64" s="131" t="inlineStr">
+      <c r="A64" s="132" t="inlineStr">
         <is>
           <t>Note 17</t>
         </is>
       </c>
-      <c r="B64" s="132" t="inlineStr">
+      <c r="B64" s="133" t="inlineStr">
         <is>
           <t>SERVICES EXTÉRIEURS</t>
         </is>
@@ -18011,7 +18020,7 @@
       <c r="H64" s="49" t="n"/>
     </row>
     <row r="65" ht="110" customHeight="1">
-      <c r="A65" s="133" t="n"/>
+      <c r="A65" s="134" t="n"/>
       <c r="B65" s="49" t="n"/>
       <c r="C65" s="49" t="n"/>
       <c r="D65" s="49" t="n"/>
@@ -18021,12 +18030,12 @@
       <c r="H65" s="49" t="n"/>
     </row>
     <row r="66" ht="16" customHeight="1">
-      <c r="A66" s="131" t="inlineStr">
+      <c r="A66" s="132" t="inlineStr">
         <is>
           <t>Note 18</t>
         </is>
       </c>
-      <c r="B66" s="132" t="inlineStr">
+      <c r="B66" s="133" t="inlineStr">
         <is>
           <t>IMPÔTS ET TAXES</t>
         </is>
@@ -18039,7 +18048,7 @@
       <c r="H66" s="49" t="n"/>
     </row>
     <row r="67" ht="110" customHeight="1">
-      <c r="A67" s="133" t="n"/>
+      <c r="A67" s="134" t="n"/>
       <c r="B67" s="49" t="n"/>
       <c r="C67" s="49" t="n"/>
       <c r="D67" s="49" t="n"/>
@@ -18049,12 +18058,12 @@
       <c r="H67" s="49" t="n"/>
     </row>
     <row r="68" ht="16" customHeight="1">
-      <c r="A68" s="131" t="inlineStr">
+      <c r="A68" s="132" t="inlineStr">
         <is>
           <t>Note 19</t>
         </is>
       </c>
-      <c r="B68" s="132" t="inlineStr">
+      <c r="B68" s="133" t="inlineStr">
         <is>
           <t>AUTRES CHARGES</t>
         </is>
@@ -18067,7 +18076,7 @@
       <c r="H68" s="49" t="n"/>
     </row>
     <row r="69" ht="110" customHeight="1">
-      <c r="A69" s="133" t="n"/>
+      <c r="A69" s="134" t="n"/>
       <c r="B69" s="49" t="n"/>
       <c r="C69" s="49" t="n"/>
       <c r="D69" s="49" t="n"/>
@@ -18082,7 +18091,7 @@
           <t>TABLE DES COMMENTAIRES</t>
         </is>
       </c>
-      <c r="G70" s="128" t="inlineStr">
+      <c r="G70" s="129" t="inlineStr">
         <is>
           <t>COMMENTAIRES
 PAGE 6/7</t>
@@ -18134,12 +18143,12 @@
       </c>
     </row>
     <row r="75" ht="16" customHeight="1">
-      <c r="A75" s="131" t="inlineStr">
+      <c r="A75" s="132" t="inlineStr">
         <is>
           <t>Note 20A</t>
         </is>
       </c>
-      <c r="B75" s="132" t="inlineStr">
+      <c r="B75" s="133" t="inlineStr">
         <is>
           <t>CHARGES DE PERSONNEL</t>
         </is>
@@ -18152,7 +18161,7 @@
       <c r="H75" s="49" t="n"/>
     </row>
     <row r="76" ht="110" customHeight="1">
-      <c r="A76" s="133" t="n"/>
+      <c r="A76" s="134" t="n"/>
       <c r="B76" s="49" t="n"/>
       <c r="C76" s="49" t="n"/>
       <c r="D76" s="49" t="n"/>
@@ -18162,12 +18171,12 @@
       <c r="H76" s="49" t="n"/>
     </row>
     <row r="77" ht="16" customHeight="1">
-      <c r="A77" s="131" t="inlineStr">
+      <c r="A77" s="132" t="inlineStr">
         <is>
           <t>Note 20B</t>
         </is>
       </c>
-      <c r="B77" s="132" t="inlineStr">
+      <c r="B77" s="133" t="inlineStr">
         <is>
           <t>EFFECTIFS, MASSE SALARIALE ET PERSONNEL EXTÉRIEUR</t>
         </is>
@@ -18180,7 +18189,7 @@
       <c r="H77" s="49" t="n"/>
     </row>
     <row r="78" ht="110" customHeight="1">
-      <c r="A78" s="133" t="n"/>
+      <c r="A78" s="134" t="n"/>
       <c r="B78" s="49" t="n"/>
       <c r="C78" s="49" t="n"/>
       <c r="D78" s="49" t="n"/>
@@ -18190,12 +18199,12 @@
       <c r="H78" s="49" t="n"/>
     </row>
     <row r="79" ht="16" customHeight="1">
-      <c r="A79" s="131" t="inlineStr">
+      <c r="A79" s="132" t="inlineStr">
         <is>
           <t>Note 21</t>
         </is>
       </c>
-      <c r="B79" s="132" t="inlineStr">
+      <c r="B79" s="133" t="inlineStr">
         <is>
           <t>CHARGES ET REVENUS FINANCIERS</t>
         </is>
@@ -18208,7 +18217,7 @@
       <c r="H79" s="49" t="n"/>
     </row>
     <row r="80" ht="110" customHeight="1">
-      <c r="A80" s="133" t="n"/>
+      <c r="A80" s="134" t="n"/>
       <c r="B80" s="49" t="n"/>
       <c r="C80" s="49" t="n"/>
       <c r="D80" s="49" t="n"/>
@@ -18218,12 +18227,12 @@
       <c r="H80" s="49" t="n"/>
     </row>
     <row r="81" ht="16" customHeight="1">
-      <c r="A81" s="131" t="inlineStr">
+      <c r="A81" s="132" t="inlineStr">
         <is>
           <t>Note 22</t>
         </is>
       </c>
-      <c r="B81" s="132" t="inlineStr">
+      <c r="B81" s="133" t="inlineStr">
         <is>
           <t>DOTATIONS ET CHARGES POUR PROVISIONS</t>
         </is>
@@ -18236,7 +18245,7 @@
       <c r="H81" s="49" t="n"/>
     </row>
     <row r="82" ht="110" customHeight="1">
-      <c r="A82" s="133" t="n"/>
+      <c r="A82" s="134" t="n"/>
       <c r="B82" s="49" t="n"/>
       <c r="C82" s="49" t="n"/>
       <c r="D82" s="49" t="n"/>
@@ -18251,7 +18260,7 @@
           <t>TABLE DES COMMENTAIRES</t>
         </is>
       </c>
-      <c r="G83" s="128" t="inlineStr">
+      <c r="G83" s="129" t="inlineStr">
         <is>
           <t>COMMENTAIRES
 PAGE 7/7</t>
@@ -18303,12 +18312,12 @@
       </c>
     </row>
     <row r="88" ht="16" customHeight="1">
-      <c r="A88" s="131" t="inlineStr">
+      <c r="A88" s="132" t="inlineStr">
         <is>
           <t>Note 23</t>
         </is>
       </c>
-      <c r="B88" s="132" t="inlineStr">
+      <c r="B88" s="133" t="inlineStr">
         <is>
           <t>AUTRES CHARGES ET PRODUITS HAO</t>
         </is>
@@ -18321,7 +18330,7 @@
       <c r="H88" s="49" t="n"/>
     </row>
     <row r="89" ht="110" customHeight="1">
-      <c r="A89" s="133" t="n"/>
+      <c r="A89" s="134" t="n"/>
       <c r="B89" s="49" t="n"/>
       <c r="C89" s="49" t="n"/>
       <c r="D89" s="49" t="n"/>
@@ -18331,12 +18340,12 @@
       <c r="H89" s="49" t="n"/>
     </row>
     <row r="90" ht="16" customHeight="1">
-      <c r="A90" s="131" t="inlineStr">
+      <c r="A90" s="132" t="inlineStr">
         <is>
           <t>Note 24</t>
         </is>
       </c>
-      <c r="B90" s="132" t="inlineStr">
+      <c r="B90" s="133" t="inlineStr">
         <is>
           <t>TABLEAU D'EXÉCUTION BUDGÉTAIRE</t>
         </is>
@@ -18349,7 +18358,7 @@
       <c r="H90" s="49" t="n"/>
     </row>
     <row r="91" ht="110" customHeight="1">
-      <c r="A91" s="133" t="n"/>
+      <c r="A91" s="134" t="n"/>
       <c r="B91" s="49" t="n"/>
       <c r="C91" s="49" t="n"/>
       <c r="D91" s="49" t="n"/>
@@ -19348,7 +19357,7 @@
       <c r="F10" s="61" t="n"/>
       <c r="G10" s="62" t="inlineStr">
         <is>
-          <t>DU : 01-01-2025    AU : 31-12-2025</t>
+          <t>DU :     AU : 31-12-2025</t>
         </is>
       </c>
       <c r="H10" s="61" t="n"/>
@@ -20464,7 +20473,7 @@
       </c>
       <c r="C9" s="5" t="n"/>
       <c r="D9" s="5">
-        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"462*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"462*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"162*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"162*",'BALANCE N'!$G$2:$G$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"462*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"462*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"162*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"162*",'BALANCE N-1'!$G$2:$G$50))+(SUMIF('BALANCE N'!$A$2:$A$50,"702*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"702*",'BALANCE N'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"162*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"162*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"462*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"462*",'BALANCE N'!$G$2:$G$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"162*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"162*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"462*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"462*",'BALANCE N-1'!$G$2:$G$50))+(SUMIF('BALANCE N'!$A$2:$A$50,"702*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"702*",'BALANCE N'!$G$2:$G$50))</f>
         <v/>
       </c>
       <c r="E9" s="71">
@@ -20521,7 +20530,7 @@
       </c>
       <c r="C12" s="5" t="n"/>
       <c r="D12" s="5">
-        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"165*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"165*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"161*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"161*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"464*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"464*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"168*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"168*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"164*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"164*",'BALANCE N'!$G$2:$G$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"165*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"165*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"161*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"161*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"464*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"464*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"168*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"168*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"164*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"164*",'BALANCE N-1'!$G$2:$G$50))</f>
+        <f>(SUMIF('BALANCE N'!$A$2:$A$50,"165*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"165*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"164*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"164*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"161*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"161*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"464*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"464*",'BALANCE N'!$G$2:$G$50)+SUMIF('BALANCE N'!$A$2:$A$50,"168*",'BALANCE N'!$H$2:$H$50)-SUMIF('BALANCE N'!$A$2:$A$50,"168*",'BALANCE N'!$G$2:$G$50))-(SUMIF('BALANCE N-1'!$A$2:$A$50,"165*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"165*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"164*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"164*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"161*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"161*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"464*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"464*",'BALANCE N-1'!$G$2:$G$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"168*",'BALANCE N-1'!$H$2:$H$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"168*",'BALANCE N-1'!$G$2:$G$50))</f>
         <v/>
       </c>
       <c r="E12" s="71">
@@ -20613,7 +20622,7 @@
         </is>
       </c>
       <c r="C16" s="5">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"231*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"233*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"232*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2391*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2392*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2393*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2396*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="D16" s="5">
@@ -20621,7 +20630,7 @@
         <v/>
       </c>
       <c r="E16" s="71">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"231*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"233*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"232*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2391*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2392*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2393*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2396*",'BALANCE N'!$H$2:$H$50)</f>
         <v/>
       </c>
     </row>
@@ -20637,7 +20646,7 @@
         </is>
       </c>
       <c r="C17" s="5">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"234*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"238*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"235*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2394*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2398*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"2395*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="D17" s="5">
@@ -20645,7 +20654,7 @@
         <v/>
       </c>
       <c r="E17" s="71">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"234*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"238*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"235*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2394*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2398*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"2395*",'BALANCE N'!$H$2:$H$50)</f>
         <v/>
       </c>
     </row>
@@ -20733,7 +20742,7 @@
         </is>
       </c>
       <c r="C21" s="5">
-        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"26*",'BALANCE N-1'!$H$2:$H$50)+SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$G$2:$G$50)-SUMIF('BALANCE N-1'!$A$2:$A$50,"27*",'BALANCE N-1'!$H$2:$H$50)</f>
         <v/>
       </c>
       <c r="D21" s="5">
@@ -20741,7 +20750,7 @@
         <v/>
       </c>
       <c r="E21" s="71">
-        <f>SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$H$2:$H$50)</f>
+        <f>SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"26*",'BALANCE N'!$H$2:$H$50)+SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$G$2:$G$50)-SUMIF('BALANCE N'!$A$2:$A$50,"27*",'BALANCE N'!$H$2:$H$50)</f>
         <v/>
       </c>
     </row>

</xml_diff>